<commit_message>
Add PDF plot exports
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="128">
   <si>
     <t xml:space="preserve">Section</t>
   </si>
@@ -279,6 +279,12 @@
   </si>
   <si>
     <t xml:space="preserve">TRUE writes cluster proportion tables and plots.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">do_pdf_plots</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRUE also saves PDF copies beside generated PNG plots.</t>
   </si>
   <si>
     <t xml:space="preserve">do_summary</t>
@@ -1252,10 +1258,24 @@
         <v>92</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>54</v>
+        <v>6</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>93</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1275,58 +1295,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1350,7 +1370,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>26</v>
@@ -1365,24 +1385,24 @@
         <v>35</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F2" s="6" t="n">
         <v>50000</v>
@@ -1390,19 +1410,19 @@
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F3" s="6" t="n">
         <v>50000</v>
@@ -1425,34 +1445,34 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>